<commit_message>
fixbug(site): update logic create & update, feat(randomization): add page randomization
</commit_message>
<xml_diff>
--- a/src/staticfiles/study/templates/event_definitions_import_template.xlsx
+++ b/src/staticfiles/study/templates/event_definitions_import_template.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -447,85 +447,80 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Study Code</t>
+          <t>Study Version</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Study Version</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Event Type</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Event Type</t>
+          <t>Phase Code</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Phase Code</t>
+          <t>Timing Mode</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Timing Mode</t>
+          <t>Sequence No</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Sequence No</t>
+          <t>Repeated</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Repeated</t>
+          <t>Max Repeats</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Max Repeats</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>Precondition</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Precondition</t>
+          <t>Day Offset</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Day Offset</t>
+          <t>Window Before Days</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Window Before Days</t>
+          <t>Window After Days</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Window After Days</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Open After Status</t>
         </is>

</xml_diff>

<commit_message>
feat(events): update full event-flows
</commit_message>
<xml_diff>
--- a/src/staticfiles/study/templates/event_definitions_import_template.xlsx
+++ b/src/staticfiles/study/templates/event_definitions_import_template.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -472,57 +472,102 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Timing Mode</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Event Category</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Execution Mode</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sequence No</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Phase Code</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Timing Mode</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Sequence No</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Repeated</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Max Repeats</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Precondition</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Day Offset</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Transition Type</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Condition Scope</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Condition Code</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Condition Expression</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Offset Days</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Window Before Days</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Window After Days</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Open After Status</t>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Auto Open</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Auto Create</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Requires Previous Completion</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Allow Skip</t>
         </is>
       </c>
     </row>

</xml_diff>